<commit_message>
Add fullflow plan and case assets
</commit_message>
<xml_diff>
--- a/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
+++ b/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\01_assist_startup_powercycle_capture`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_163604_yichang_formal_fullflow_r1\03_execution\steps\01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -636,8 +636,8 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\02_burn\burn.log`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\01_assist_startup_powercycle_capture`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_163604_yichang_formal_fullflow_r1\02_burn\burn.log`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_163604_yichang_formal_fullflow_r1\03_execution\steps\01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -696,7 +696,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\01_assist_startup_powercycle_capture`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_163604_yichang_formal_fullflow_r1\03_execution\steps\01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -782,7 +782,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>唤醒超时退出与休息语（需求 `20s`）</t>
+          <t>唤醒超时退出与休息语（需求 `15s`）</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -988,8 +988,8 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\13_sess_exit_sequence_only`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\14_sess_exit_rewake_open_recovery`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\28_sess_exit_sequence_only`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\29_sess_exit_rewake_open_recovery`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\12_sess_idle_open_blocked`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\27_sess_idle_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1421,7 +1421,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>音量设置不应掉电保存（需求默认音量 `4`）</t>
+          <t>音量设置应掉电保存（需求保持断电前档位）</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1438,12 +1438,12 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>重启后应恢复需求默认音量，而不是保留断电前档位</t>
+          <t>重启后应保持断电前音量档位，不应恢复成其他值</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>`COM38` 启动日志中的 `volume` 与重启后行为应回到默认值</t>
+          <t>`COM38` 启动日志中的 `volume` 与重启后行为应保持断电前档位</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
@@ -1453,8 +1453,8 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\08_cfg_volume_nonpersist_min`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\09_cfg_volume_nonpersist_reboot`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\23_cfg_volume_persist_probe_min`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\24_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\15_volume_rapid_stability`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\30_volume_rapid_stability`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1927,8 +1927,8 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\19_voice_valid_proto_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\20_voice_on_then_volume_up`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\34_voice_valid_proto_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\35_voice_on_then_volume_up`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2048,9 +2048,9 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\16_assist_voice_off_setup`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\17_voice_invalid_proto`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\18_voice_invalid_proto_then_wake_open_blocked`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\31_assist_voice_off_setup`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\32_voice_invalid_proto`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\33_voice_invalid_proto_then_wake_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2223,9 +2223,9 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\21_switch_wake_to_next`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\30_switch_idle_before_other_wake_blocked`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\31_switch_other_wake_blocked`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\36_switch_wake_to_next`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\45_switch_idle_before_other_wake_blocked`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\46_switch_other_wake_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2285,11 +2285,11 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\21_switch_wake_to_next`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\22_switch_idle_before_current_wake_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\23_switch_current_wake_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\24_switch_idle_before_current_wake_volume`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\25_switch_current_wake_volume`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\36_switch_wake_to_next`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\37_switch_idle_before_current_wake_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\38_switch_current_wake_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\39_switch_idle_before_current_wake_volume`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\40_switch_current_wake_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2349,11 +2349,11 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\21_switch_wake_to_next`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\26_switch_idle_before_default_wake_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\27_switch_default_wake_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\28_switch_idle_before_default_wake_volume`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\29_switch_default_wake_volume`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\36_switch_wake_to_next`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\41_switch_idle_before_default_wake_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\42_switch_default_wake_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\43_switch_idle_before_default_wake_volume`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\44_switch_default_wake_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2471,11 +2471,11 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\21_switch_wake_to_next`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\32_switch_cycle_to_tmall`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\33_switch_idle_before_tmall_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\34_switch_cycle_tmall_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\35_switch_cycle_back_default`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\36_switch_wake_to_next`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\47_switch_cycle_to_tmall`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\48_switch_idle_before_tmall_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\49_switch_cycle_tmall_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\50_switch_cycle_back_default`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2648,9 +2648,9 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\38_reg_entry_timeout_wait30s`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\39_reg_entry_timeout_idle_30s`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\40_reg_entry_timeout_recover_open`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\53_reg_entry_timeout_wait30s`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\54_reg_entry_timeout_idle_30s`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\55_reg_entry_timeout_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2885,9 +2885,9 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\41_reg_cmd_learn_close_sequence`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\42_reg_cmd_alias_close_recheck`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\43_reg_cmd_default_close_recheck`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\56_reg_cmd_learn_close_sequence`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\57_reg_cmd_alias_close_recheck`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\58_reg_cmd_default_close_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3063,9 +3063,9 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\46_reg_wake_learn_sequence`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\48_reg_wake_newword_open`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\49_reg_wake_newword_volume`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\61_reg_wake_learn_sequence`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\63_reg_wake_newword_open`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\64_reg_wake_newword_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3123,9 +3123,9 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\46_reg_wake_learn_sequence`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\50_reg_wake_idle_before_other_ordinary_blocked`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\51_reg_wake_other_ordinary_blocked`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\61_reg_wake_learn_sequence`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\65_reg_wake_idle_before_other_ordinary_blocked`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\66_reg_wake_other_ordinary_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3307,9 +3307,9 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\54_powerloss_during_case_enter_learning`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\55_powerloss_during_case_boot`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\56_powerloss_during_case_recover_open`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\69_powerloss_during_case_enter_learning`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\70_powerloss_during_case_boot`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\71_powerloss_during_case_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3608,8 +3608,8 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418072549_26_reg_voice007_cmd_conflict_volume_word_sequence`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418072637_27_reg_voice007_cmd_conflict_volume_word_recheck`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\83_reg_conflict_cmd_volume_word_sequence`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\84_reg_conflict_cmd_volume_word_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4074,14 +4074,14 @@
           <t>辅助看 `AGAIN=36dB`、`DGAIN=6dB`</t>
         </is>
       </c>
-      <c r="J61" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J61" s="4" t="inlineStr">
+        <is>
+          <t>TODO</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\04_assist_reboot_after_config_clear`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4109,7 +4109,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>唤醒会话时长应为 `20s`</t>
+          <t>唤醒会话时长应为 `15s`</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4126,7 +4126,7 @@
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>会话超时应接近并满足需求 `20s`</t>
+          <t>会话超时应接近并满足需求 `15s`</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -4134,14 +4134,16 @@
           <t>`COM38` 辅助看 `MODE=1`、`TIME_OUT`、`MODE=0` 及回收时间</t>
         </is>
       </c>
-      <c r="J62" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\041717_timeout_then_open_fan_dual_retry\meta.json`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\07_cfg_wake_timeout_probe`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\08_cfg_wake_timeout_probe_settle`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\09_cfg_wake_timeout_post_command_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4169,7 +4171,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>默认音量应为 `4`</t>
+          <t>默认音量应为 `3`</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -4185,7 +4187,7 @@
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>默认音量字段应为 `4`</t>
+          <t>默认音量字段应为 `3`</t>
         </is>
       </c>
       <c r="I63" s="2" t="inlineStr">
@@ -4200,7 +4202,7 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\04_assist_reboot_after_config_clear`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4228,7 +4230,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>音量总档位应为 `6`</t>
+          <t>音量总档位应为 `5`</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4244,7 +4246,7 @@
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>应存在连续 `6` 个有效档位</t>
+          <t>应存在连续 `5` 个有效档位</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr">
@@ -4252,16 +4254,27 @@
           <t>可辅助看 `refresh config volume=`、边界 tone 与控制效果</t>
         </is>
       </c>
-      <c r="J64" s="5" t="inlineStr">
-        <is>
-          <t>FAIL</t>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418164815_fullflow_volume_rapid_stability\log_utf8.txt`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\04180012_reg_volume_max_powercycle_boot\boot_log_utf8.txt`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\04180016_reg_volume_min_powercycle_boot\boot_log_utf8.txt`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\11_cfg_volume_level_probe_min_anchor`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\12_cfg_volume_level_probe_up_1`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\13_cfg_volume_level_probe_up_2`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\14_cfg_volume_level_probe_up_3`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\15_cfg_volume_level_probe_up_4`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\16_cfg_volume_level_probe_up_5`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\17_cfg_volume_level_probe_max_anchor`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\18_cfg_volume_level_probe_down_1`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\19_cfg_volume_level_probe_down_2`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\20_cfg_volume_level_probe_down_3`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\21_cfg_volume_level_probe_down_4`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\22_cfg_volume_level_probe_down_5`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\23_cfg_volume_persist_probe_min`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\24_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4320,7 +4333,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\14_sess_exit_rewake_open_recovery`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\29_sess_exit_rewake_open_recovery`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4380,8 +4393,8 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\16_assist_voice_off_setup`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\03_execution\steps\19_voice_valid_proto_open`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\31_assist_voice_off_setup`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\34_voice_valid_proto_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4440,7 +4453,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\041717_passive_report_baseline_after_release\log_utf8.txt`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\10_cfg_passive_report_proto`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4492,14 +4505,14 @@
           <t>辅助看 `reg again!` 次数与学习收口</t>
         </is>
       </c>
-      <c r="J68" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418071510_03_reg_tc_learn_cmd_close_sequence\log_utf8.txt`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\56_reg_cmd_learn_close_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4551,14 +4564,14 @@
           <t>辅助看 `reg again!` 次数与学习收口</t>
         </is>
       </c>
-      <c r="J69" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418073052_37_reg_voice002_learn_wakeup_sequence\log_utf8.txt`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\61_reg_wake_learn_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4610,15 +4623,15 @@
           <t>辅助看 `reg simila error!`、`error cnt &gt; N`、`reg failed!`</t>
         </is>
       </c>
-      <c r="J70" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J70" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418072345_22_reg_voice005_cmd_retry_exhaust_sequence\log_utf8.txt`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418072503_23_reg_voice005_cmd_retry_exhaust_failed_alias_probe`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\74_reg_cfg_cmd_retry_exhaust_sequence`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\75_reg_cfg_cmd_retry_exhaust_failed_alias_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4670,15 +4683,16 @@
           <t>辅助看 `reg simila error!`、`error cnt &gt; N`、`reg failed!`</t>
         </is>
       </c>
-      <c r="J71" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418073824_54_reg_voice006_wakeup_retry_exhaust_sequence\log_utf8.txt`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418073938_55_reg_voice006_wakeup_retry_exhaust_failed_wake_probe`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\78_reg_cfg_wake_retry_exhaust_sequence`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\79_reg_cfg_wake_retry_exhaust_failed_wake_probe`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\80_reg_cfg_wake_retry_exhaust_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4730,15 +4744,15 @@
           <t>辅助看 `regCmdCount`、`reg over!` 等日志</t>
         </is>
       </c>
-      <c r="J72" s="3" t="inlineStr">
-        <is>
-          <t>PASS</t>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\04172315_powercycle_boot_log\boot_log_utf8.txt`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\04180018_reg_learn_entry_exit_default_open\log_utf8.txt`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\01_assist_startup_powercycle_capture`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\04_assist_reg_cmd_template_full_entry`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4797,8 +4811,9 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\0418073052_37_reg_voice002_learn_wakeup_sequence\log_utf8.txt`
-`deliverables\csk5062_xiaodu_fan\reports\20260419_162517_post_restructure_fullflow\04_preserved_result_refs\result\04172212_wakeup_reserved_learn_cmd_word\log_utf8.txt`
+          <t>`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\61_reg_wake_learn_sequence`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\62_reg_wake_template_full_reenter`
+`deliverables\csk5062_xiaodu_fan\reports\20260420_160258_xieyierror_formal_fullflow_r1\03_execution\steps\63_reg_wake_newword_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4850,7 +4865,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
@@ -4860,7 +4875,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -4870,7 +4885,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
feat: publish reusable fullflow validation skill
</commit_message>
<xml_diff>
--- a/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
+++ b/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
@@ -585,7 +585,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -644,8 +644,8 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/02_burn/burn.log`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/02_burn/burn.log`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -704,7 +704,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -763,7 +763,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/03_sess_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/03_sess_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -822,7 +822,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/04_sess_timeout_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/04_sess_timeout_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -881,8 +881,8 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/04_sess_timeout_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/05_sess_timeout_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/04_sess_timeout_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/05_sess_timeout_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -941,7 +941,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/06_sess_exit_then_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/06_sess_exit_then_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1000,8 +1000,8 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/45_sess_exit_sequence_only`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/46_sess_exit_rewake_open_recovery`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/45_sess_exit_sequence_only`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/46_sess_exit_rewake_open_recovery`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1060,7 +1060,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/44_sess_idle_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/44_sess_idle_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/03_sess_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/03_sess_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1176,7 +1176,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/07_ctrl_close`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/07_ctrl_close`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1234,7 +1234,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/08_ctrl_power_on`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/08_ctrl_power_on`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/09_ctrl_power_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/09_ctrl_power_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/10_vol_up_down`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/10_vol_up_down`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1410,8 +1410,8 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/11_vol_max`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/12_vol_min`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/11_vol_max`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/12_vol_min`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1471,9 +1471,9 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/39_cfg_volume_persist_probe_min`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/40_cfg_volume_persist_wait_refresh`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/41_cfg_volume_powercycle_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/39_cfg_volume_persist_probe_min`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/40_cfg_volume_persist_wait_refresh`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/41_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/47_volume_rapid_stability`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/47_volume_rapid_stability`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1591,8 +1591,8 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/16_report_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/17_report_off_then_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/16_report_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/17_report_off_then_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1651,9 +1651,9 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/15_report_passive_baseline`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/16_report_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/18_report_passive_after_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/15_report_passive_baseline`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/16_report_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/18_report_passive_after_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1713,9 +1713,9 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/19_report_on_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/20_report_on_then_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/21_report_passive_after_on`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/19_report_on_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/20_report_on_then_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/21_report_passive_after_on`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1774,9 +1774,9 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/22_report_off_before_powercycle`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/23_report_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/24_report_after_powercycle_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/22_report_off_before_powercycle`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/23_report_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/24_report_after_powercycle_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1835,8 +1835,8 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/27_voice_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/28_voice_blocked_after_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/27_voice_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/28_voice_blocked_after_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1895,8 +1895,8 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/31_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/32_voice_open_after_proto`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/31_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/32_voice_open_after_proto`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1955,8 +1955,8 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/51_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/52_voice_on_then_volume_up`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/51_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/52_voice_on_then_volume_up`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2015,12 +2015,12 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/27_voice_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/29_voice_off_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/30_voice_blocked_after_powercycle`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/31_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/33_voice_on_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/34_voice_open_after_powercycle`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/27_voice_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/29_voice_off_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/30_voice_blocked_after_powercycle`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/31_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/33_voice_on_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/34_voice_open_after_powercycle`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2079,9 +2079,9 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/48_assist_voice_off_setup`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/49_voice_invalid_proto`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/50_voice_invalid_proto_then_wake_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/48_assist_voice_off_setup`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/49_voice_invalid_proto`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/50_voice_invalid_proto_then_wake_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2140,9 +2140,9 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/38_switch_idle_before_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/39_switch_xiaoai_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/38_switch_idle_before_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/39_switch_xiaoai_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2200,9 +2200,9 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/40_switch_idle_before_default`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/41_switch_default_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/40_switch_idle_before_default`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/41_switch_default_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2260,9 +2260,9 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/62_switch_idle_before_other_wake_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/63_switch_other_wake_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/62_switch_idle_before_other_wake_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/63_switch_other_wake_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2322,11 +2322,11 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/54_switch_idle_before_current_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/55_switch_current_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/56_switch_idle_before_current_wake_volume`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/57_switch_current_wake_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/54_switch_idle_before_current_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/55_switch_current_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/56_switch_idle_before_current_wake_volume`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/57_switch_current_wake_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2386,13 +2386,13 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/01_closure_swake005_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/02_closure_swake005_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/03_closure_swake005_switch_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/04_closure_swake005_idle_before_default_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/05_closure_swake005_default_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/06_closure_swake005_idle_before_default_volume`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/07_closure_swake005_default_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/01_closure_swake005_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/02_closure_swake005_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/03_closure_swake005_switch_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/04_closure_swake005_idle_before_default_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/05_closure_swake005_default_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/06_closure_swake005_idle_before_default_volume`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/07_closure_swake005_default_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2451,12 +2451,12 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/42_switch_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/43_switch_idle_before_xiaoai_after_power`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/44_switch_xiaoai_after_power_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/45_switch_idle_before_default_after_power`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/46_switch_default_after_power_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/42_switch_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/43_switch_idle_before_xiaoai_after_power`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/44_switch_xiaoai_after_power_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/45_switch_idle_before_default_after_power`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/46_switch_default_after_power_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2515,11 +2515,11 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/64_switch_cycle_to_tmall`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/65_switch_idle_before_tmall_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/66_switch_cycle_tmall_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/67_switch_cycle_back_default`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/64_switch_cycle_to_tmall`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/65_switch_idle_before_tmall_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/66_switch_cycle_tmall_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/67_switch_cycle_back_default`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2577,7 +2577,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/49_reg_entry_cmd_only`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/49_reg_entry_cmd_only`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/56_reg_entry_wake_only`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/56_reg_entry_wake_only`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2694,9 +2694,9 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/70_reg_entry_timeout_wait30s`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/71_reg_entry_timeout_idle_30s`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/72_reg_entry_timeout_recover_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/70_reg_entry_timeout_wait30s`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/71_reg_entry_timeout_idle_30s`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/72_reg_entry_timeout_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2755,8 +2755,8 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/52_reg_exit_learning_then_recover`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_223038_linux_missing_nonreg_merge_r1/03_execution/steps/53_reg_exit_default_open_recover`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/52_reg_exit_learning_then_recover`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/53_reg_exit_default_open_recover`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2815,15 +2815,15 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2882,15 +2882,15 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2949,15 +2949,15 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3016,9 +3016,9 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/82_reg_wake_newword_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/83_reg_wake_newword_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/82_reg_wake_newword_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/83_reg_wake_newword_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3076,8 +3076,8 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225152_38_reg_voice002_learn_wakeup_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225222_40_reg_voice002_default_wake_still_open_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120717_38_reg_voice002_learn_wakeup_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120751_40_reg_voice002_default_wake_still_open_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3137,9 +3137,9 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/82_reg_wake_newword_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/83_reg_wake_newword_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/82_reg_wake_newword_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/83_reg_wake_newword_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3197,9 +3197,9 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/84_reg_wake_idle_before_other_ordinary_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/85_reg_wake_other_ordinary_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/84_reg_wake_idle_before_other_ordinary_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/85_reg_wake_other_ordinary_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3259,8 +3259,8 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225028_34_reg_tc_learn_prev_boundary`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225058_35_reg_tc_learn_next_boundary_full`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120559_34_reg_tc_learn_prev_boundary`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120629_35_reg_tc_learn_next_boundary_full`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3320,11 +3320,11 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225907_67_reg_tc_learn003_learn_wakeup_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225931_68_reg_tc_learn003_learn_cmd_full_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424230000_69_reg_tc_learn003_pre_powercycle_recheck`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424230029_70_reg_tc_learn003_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424230049_71_reg_tc_learn003_post_powercycle_recheck`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121436_67_reg_tc_learn003_learn_wakeup_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121459_68_reg_tc_learn003_learn_cmd_full_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121528_69_reg_tc_learn003_pre_powercycle_recheck`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121558_70_reg_tc_learn003_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121617_71_reg_tc_learn003_post_powercycle_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3383,9 +3383,9 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/88_powerloss_during_case_enter_learning`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/89_powerloss_during_case_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/90_powerloss_during_case_recover_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/88_powerloss_during_case_enter_learning`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/89_powerloss_during_case_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/90_powerloss_during_case_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3445,8 +3445,8 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224618_19_reg_voice003_cmd_retry_recover_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224654_20_reg_voice003_cmd_retry_recover_alias_recheck`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120149_19_reg_voice003_cmd_retry_recover_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120225_20_reg_voice003_cmd_retry_recover_alias_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3505,9 +3505,9 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225456_51_reg_voice004_wakeup_retry_recover_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225528_52_reg_voice004_wakeup_retry_recover_recheck_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225539_53_reg_voice004_wakeup_retry_recover_default_wake_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121024_51_reg_voice004_wakeup_retry_recover_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121056_52_reg_voice004_wakeup_retry_recover_recheck_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121107_53_reg_voice004_wakeup_retry_recover_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3566,8 +3566,8 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224727_23_reg_voice005_cmd_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224812_24_reg_voice005_cmd_retry_exhaust_failed_alias_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120258_23_reg_voice005_cmd_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120343_24_reg_voice005_cmd_retry_exhaust_failed_alias_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3626,9 +3626,9 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/97_reg_cfg_wake_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/98_reg_cfg_wake_retry_exhaust_failed_wake_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/99_reg_cfg_wake_retry_exhaust_default_wake_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/97_reg_cfg_wake_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/98_reg_cfg_wake_retry_exhaust_failed_wake_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/99_reg_cfg_wake_retry_exhaust_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3687,9 +3687,9 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/102_reg_conflict_cmd_volume_word_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/103_reg_conflict_reboot_after_attempt`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/104_reg_conflict_cmd_volume_word_recheck`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/102_reg_conflict_cmd_volume_word_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/103_reg_conflict_reboot_after_attempt`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/104_reg_conflict_cmd_volume_word_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3747,9 +3747,9 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/25_closure_conflict_default_wake_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/26_closure_conflict_default_wake_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/27_closure_conflict_default_wake_sequence`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/25_closure_conflict_default_wake_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/26_closure_conflict_default_wake_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/27_closure_conflict_default_wake_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224943_31_reg_voice009_cmd_reserved_learn_wakeup_word`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120514_31_reg_voice009_cmd_reserved_learn_wakeup_word`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225820_64_reg_voice010_wakeup_reserved_learn_cmd_word`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121349_64_reg_voice010_wakeup_reserved_learn_cmd_word`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3925,9 +3925,9 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224422_10_reg_delete_cmd_confirm_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224437_11_reg_delete_cmd_confirm_alias_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424224448_12_reg_delete_cmd_confirm_default_close_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426115953_10_reg_delete_cmd_confirm_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120008_11_reg_delete_cmd_confirm_alias_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120019_12_reg_delete_cmd_confirm_default_close_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3987,17 +3987,17 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/18_closure_regcmd_delete_exit_keep`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230959_fresh_closure_targets_merge_r1/03_execution/steps/19_closure_regcmd_alias_after_delete_exit`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/18_closure_regcmd_delete_exit_keep`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/19_closure_regcmd_alias_after_delete_exit`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4057,10 +4057,10 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225330_45_reg_voice013_delete_wakeup_confirm_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225350_46_reg_voice013_delete_wakeup_confirm_reboot_after_delete`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225408_47_reg_voice013_delete_wakeup_confirm_learned_wake_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225422_48_reg_voice013_delete_wakeup_confirm_default_wake_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120859_45_reg_voice013_delete_wakeup_confirm_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120918_46_reg_voice013_delete_wakeup_confirm_reboot_after_delete`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120936_47_reg_voice013_delete_wakeup_confirm_learned_wake_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120951_48_reg_voice013_delete_wakeup_confirm_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4120,8 +4120,8 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225303_43_reg_voice014_delete_wakeup_exit_keep`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_224158_linux_voice_reg_batch_merge_r1/steps/0424225319_44_reg_voice014_delete_wakeup_exit_keep_recheck`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120831_43_reg_voice014_delete_wakeup_exit_keep`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120848_44_reg_voice014_delete_wakeup_exit_keep_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4180,7 +4180,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4240,8 +4240,8 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_230627_timeout_volume_probe_merge_r1/03_execution/steps/04_probe_wake_only_timeout`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_230627_timeout_volume_probe_merge_r1/03_execution/steps/06_probe_wake_cmd_timeout`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_121800_two_req_xiaodu_timeout_volume_r1/03_execution/steps/04_probe_wake_only_timeout`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_121800_two_req_xiaodu_timeout_volume_r1/03_execution/steps/06_probe_wake_cmd_timeout`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4302,21 +4302,21 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/01_assist_startup_powercycle_capture`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/04_cfg_default_volume_position_probe_default_to_max_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/05_cfg_default_volume_position_probe_default_to_max_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/06_cfg_default_volume_position_probe_default_to_max_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/07_cfg_default_volume_position_probe_default_to_max_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/08_cfg_default_volume_position_probe_max_to_min_down_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/09_cfg_default_volume_position_probe_max_to_min_down_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/10_cfg_default_volume_position_probe_max_to_min_down_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/11_cfg_default_volume_position_probe_max_to_min_down_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/12_cfg_default_volume_position_probe_max_to_min_down_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/13_cfg_default_volume_position_probe_min_to_max_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/14_cfg_default_volume_position_probe_min_to_max_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/15_cfg_default_volume_position_probe_min_to_max_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/16_cfg_default_volume_position_probe_min_to_max_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/17_cfg_default_volume_position_probe_min_to_max_up_5`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/04_cfg_default_volume_position_probe_default_to_max_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/05_cfg_default_volume_position_probe_default_to_max_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/06_cfg_default_volume_position_probe_default_to_max_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/07_cfg_default_volume_position_probe_default_to_max_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/08_cfg_default_volume_position_probe_max_to_min_down_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/09_cfg_default_volume_position_probe_max_to_min_down_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/10_cfg_default_volume_position_probe_max_to_min_down_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/11_cfg_default_volume_position_probe_max_to_min_down_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/12_cfg_default_volume_position_probe_max_to_min_down_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/13_cfg_default_volume_position_probe_min_to_max_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/14_cfg_default_volume_position_probe_min_to_max_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/15_cfg_default_volume_position_probe_min_to_max_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/16_cfg_default_volume_position_probe_min_to_max_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/17_cfg_default_volume_position_probe_min_to_max_up_5`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4375,21 +4375,21 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/27_cfg_volume_level_probe_min_anchor`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/28_cfg_volume_level_probe_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/29_cfg_volume_level_probe_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/30_cfg_volume_level_probe_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/31_cfg_volume_level_probe_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/32_cfg_volume_level_probe_up_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/33_cfg_volume_level_probe_max_anchor`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/34_cfg_volume_level_probe_down_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/35_cfg_volume_level_probe_down_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/36_cfg_volume_level_probe_down_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/37_cfg_volume_level_probe_down_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/38_cfg_volume_level_probe_down_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/39_cfg_volume_persist_probe_min`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/40_cfg_volume_persist_wait_refresh`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/41_cfg_volume_powercycle_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/27_cfg_volume_level_probe_min_anchor`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/28_cfg_volume_level_probe_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/29_cfg_volume_level_probe_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/30_cfg_volume_level_probe_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/31_cfg_volume_level_probe_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/32_cfg_volume_level_probe_up_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/33_cfg_volume_level_probe_max_anchor`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/34_cfg_volume_level_probe_down_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/35_cfg_volume_level_probe_down_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/36_cfg_volume_level_probe_down_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/37_cfg_volume_level_probe_down_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/38_cfg_volume_level_probe_down_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/39_cfg_volume_persist_probe_min`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/40_cfg_volume_persist_wait_refresh`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/41_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4448,7 +4448,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/03_assist_gate_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/03_assist_gate_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4508,8 +4508,8 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/48_assist_voice_off_setup`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/51_voice_valid_proto_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/48_assist_voice_off_setup`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/51_voice_valid_proto_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4568,7 +4568,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/26_cfg_passive_report_proto`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/26_cfg_passive_report_proto`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/73_reg_cmd_learn_close_sequence`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/73_reg_cmd_learn_close_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4686,7 +4686,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/80_reg_wake_learn_sequence`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4745,8 +4745,8 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/93_reg_cfg_cmd_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/94_reg_cfg_cmd_retry_exhaust_failed_alias_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/93_reg_cfg_cmd_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/94_reg_cfg_cmd_retry_exhaust_failed_alias_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4805,9 +4805,9 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/97_reg_cfg_wake_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/98_reg_cfg_wake_retry_exhaust_failed_wake_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/99_reg_cfg_wake_retry_exhaust_default_wake_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/97_reg_cfg_wake_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/98_reg_cfg_wake_retry_exhaust_failed_wake_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/99_reg_cfg_wake_retry_exhaust_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4867,8 +4867,8 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/01_assist_startup_powercycle_capture`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/20_assist_reg_cmd_template_full_entry`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/20_assist_reg_cmd_template_full_entry`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4927,9 +4927,9 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/81_reg_wake_template_full_reenter`
-`deliverables/csk5062_xiaodu_fan/reports/20260424_182524_linux_acm_fullflow_merge_r2/03_execution/steps/82_reg_wake_newword_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/81_reg_wake_template_full_reenter`
+`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/82_reg_wake_newword_open`
 目录重构后复跑闭环</t>
         </is>
       </c>

</xml_diff>

<commit_message>
feat: add unified formal suite runner
</commit_message>
<xml_diff>
--- a/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
+++ b/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
@@ -30,7 +30,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -52,11 +52,6 @@
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9EAF7"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -70,7 +65,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -85,9 +80,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -470,7 +462,7 @@
     <col width="43" customWidth="1" min="7" max="7"/>
     <col width="49" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
     <col width="60" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -585,7 +577,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -644,8 +636,8 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/02_burn/burn.log`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/02_burn/burn.log`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -704,7 +696,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -763,7 +755,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/03_sess_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/03_sess_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -822,7 +814,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/04_sess_timeout_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/04_sess_timeout_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -881,8 +873,8 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/04_sess_timeout_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/05_sess_timeout_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/04_sess_timeout_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/05_sess_timeout_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -941,7 +933,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/06_sess_exit_then_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/06_sess_exit_then_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1000,8 +992,8 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/45_sess_exit_sequence_only`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/46_sess_exit_rewake_open_recovery`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/45_sess_exit_sequence_only`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/46_sess_exit_rewake_open_recovery`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1060,7 +1052,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/44_sess_idle_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/44_sess_idle_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1118,7 +1110,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/03_sess_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/03_sess_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1176,7 +1168,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/07_ctrl_close`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/07_ctrl_close`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1234,7 +1226,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/08_ctrl_power_on`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/08_ctrl_power_on`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1292,7 +1284,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/09_ctrl_power_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/09_ctrl_power_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1351,7 +1343,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/10_vol_up_down`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/10_vol_up_down`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1410,8 +1402,8 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/11_vol_max`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/12_vol_min`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/11_vol_max`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/12_vol_min`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1471,9 +1463,9 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/39_cfg_volume_persist_probe_min`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/40_cfg_volume_persist_wait_refresh`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/41_cfg_volume_powercycle_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/39_cfg_volume_persist_probe_min`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/40_cfg_volume_persist_wait_refresh`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/41_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1532,7 +1524,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/47_volume_rapid_stability`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/47_volume_rapid_stability`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1591,8 +1583,8 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/16_report_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/17_report_off_then_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/16_report_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/17_report_off_then_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1651,9 +1643,9 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/15_report_passive_baseline`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/16_report_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/18_report_passive_after_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/15_report_passive_baseline`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/16_report_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/18_report_passive_after_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1713,9 +1705,9 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/19_report_on_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/20_report_on_then_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/21_report_passive_after_on`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/19_report_on_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/20_report_on_then_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/21_report_passive_after_on`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1774,9 +1766,9 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/22_report_off_before_powercycle`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/23_report_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/24_report_after_powercycle_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/22_report_off_before_powercycle`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/23_report_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/24_report_after_powercycle_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1835,8 +1827,8 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/27_voice_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/28_voice_blocked_after_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/27_voice_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/28_voice_blocked_after_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1895,8 +1887,8 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/31_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/32_voice_open_after_proto`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/31_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/32_voice_open_after_proto`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1955,8 +1947,8 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/51_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/52_voice_on_then_volume_up`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/51_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/52_voice_on_then_volume_up`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2015,12 +2007,12 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/27_voice_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/29_voice_off_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/30_voice_blocked_after_powercycle`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/31_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/33_voice_on_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/34_voice_open_after_powercycle`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/27_voice_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/29_voice_off_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/30_voice_blocked_after_powercycle`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/31_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/33_voice_on_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/34_voice_open_after_powercycle`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2079,9 +2071,9 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/48_assist_voice_off_setup`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/49_voice_invalid_proto`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/50_voice_invalid_proto_then_wake_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/48_assist_voice_off_setup`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/49_voice_invalid_proto`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/50_voice_invalid_proto_then_wake_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2140,9 +2132,9 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/38_switch_idle_before_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/39_switch_xiaoai_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/38_switch_idle_before_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/39_switch_xiaoai_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2200,9 +2192,9 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/40_switch_idle_before_default`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/41_switch_default_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/40_switch_idle_before_default`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/41_switch_default_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2260,9 +2252,9 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/62_switch_idle_before_other_wake_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/63_switch_other_wake_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/62_switch_idle_before_other_wake_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/63_switch_other_wake_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2322,11 +2314,11 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/54_switch_idle_before_current_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/55_switch_current_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/56_switch_idle_before_current_wake_volume`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/57_switch_current_wake_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/54_switch_idle_before_current_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/55_switch_current_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/56_switch_idle_before_current_wake_volume`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/57_switch_current_wake_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2386,13 +2378,11 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/01_closure_swake005_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/02_closure_swake005_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/03_closure_swake005_switch_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/04_closure_swake005_idle_before_default_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/05_closure_swake005_default_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/06_closure_swake005_idle_before_default_volume`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/07_closure_swake005_default_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/58_switch_idle_before_default_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/59_switch_default_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/60_switch_idle_before_default_wake_volume`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/61_switch_default_wake_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2451,12 +2441,12 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/42_switch_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/43_switch_idle_before_xiaoai_after_power`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/44_switch_xiaoai_after_power_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/45_switch_idle_before_default_after_power`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/46_switch_default_after_power_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/42_switch_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/43_switch_idle_before_xiaoai_after_power`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/44_switch_xiaoai_after_power_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/45_switch_idle_before_default_after_power`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/46_switch_default_after_power_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2515,11 +2505,11 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/64_switch_cycle_to_tmall`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/65_switch_idle_before_tmall_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/66_switch_cycle_tmall_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/67_switch_cycle_back_default`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/64_switch_cycle_to_tmall`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/65_switch_idle_before_tmall_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/66_switch_cycle_tmall_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/67_switch_cycle_back_default`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2577,7 +2567,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/49_reg_entry_cmd_only`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/49_reg_entry_cmd_only`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2635,7 +2625,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/56_reg_entry_wake_only`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/56_reg_entry_wake_only`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2694,9 +2684,9 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/70_reg_entry_timeout_wait30s`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/71_reg_entry_timeout_idle_30s`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/72_reg_entry_timeout_recover_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/71_reg_entry_timeout_wait30s`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/72_reg_entry_timeout_idle_30s`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/73_reg_entry_timeout_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2755,8 +2745,8 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/52_reg_exit_learning_then_recover`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_114510_two_req_xiaodu_missing_r1/03_execution/steps/53_reg_exit_default_open_recover`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/52_reg_exit_learning_then_recover`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/53_reg_exit_default_open_recover`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2815,15 +2805,10 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
+          <t>`result/csk5062_xiaodu_fan/0429225133_03_reg_tc_learn_cmd_close_sequence`
+`result/csk5062_xiaodu_fan/0429225206_04_reg_tc_learn_cmd_close_save_closure`
+`result/csk5062_xiaodu_fan/0429225223_05_reg_tc_learn_cmd_close_persist_reboot`
+`result/csk5062_xiaodu_fan/0429225241_06_reg_tc_learn_cmd_close_alias_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2882,15 +2867,10 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
+          <t>`result/csk5062_xiaodu_fan/0429225133_03_reg_tc_learn_cmd_close_sequence`
+`result/csk5062_xiaodu_fan/0429225206_04_reg_tc_learn_cmd_close_save_closure`
+`result/csk5062_xiaodu_fan/0429225223_05_reg_tc_learn_cmd_close_persist_reboot`
+`result/csk5062_xiaodu_fan/0429225252_07_reg_tc_learn_cmd_close_after_reboot_alias`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2949,15 +2929,11 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/74_reg_cmd_learn_close_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/75_reg_cmd_learn_close_save_closure`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/76_reg_cmd_reboot_after_save`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/77_reg_cmd_alias_close_recheck`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/78_reg_cmd_default_close_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3016,9 +2992,8 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/82_reg_wake_newword_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/83_reg_wake_newword_volume`
+          <t>`result/csk5062_xiaodu_fan/0429230044_38_reg_voice002_learn_wakeup_sequence`
+`result/csk5062_xiaodu_fan/0429230106_39_reg_voice002_learned_wake_recheck_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3076,8 +3051,8 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120717_38_reg_voice002_learn_wakeup_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120751_40_reg_voice002_default_wake_still_open_ok`
+          <t>`result/csk5062_xiaodu_fan/0429230044_38_reg_voice002_learn_wakeup_sequence`
+`result/csk5062_xiaodu_fan/0429230117_40_reg_voice002_default_wake_still_open_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3137,9 +3112,9 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/82_reg_wake_newword_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/83_reg_wake_newword_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/83_reg_wake_newword_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/84_reg_wake_newword_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3197,9 +3172,9 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/84_reg_wake_idle_before_other_ordinary_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/85_reg_wake_other_ordinary_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/85_reg_wake_idle_before_other_ordinary_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/86_reg_wake_other_ordinary_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3259,8 +3234,8 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120559_34_reg_tc_learn_prev_boundary`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120629_35_reg_tc_learn_next_boundary_full`
+          <t>`result/csk5062_xiaodu_fan/0429225935_34_reg_tc_learn_prev_boundary`
+`result/csk5062_xiaodu_fan/0429225957_35_reg_tc_learn_next_boundary_full`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3320,11 +3295,11 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121436_67_reg_tc_learn003_learn_wakeup_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121459_68_reg_tc_learn003_learn_cmd_full_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121528_69_reg_tc_learn003_pre_powercycle_recheck`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121558_70_reg_tc_learn003_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121617_71_reg_tc_learn003_post_powercycle_recheck`
+          <t>`result/csk5062_xiaodu_fan/0429230818_68_reg_tc_learn003_learn_wakeup_sequence`
+`result/csk5062_xiaodu_fan/0429230841_69_reg_tc_learn003_learn_cmd_full_sequence`
+`result/csk5062_xiaodu_fan/0429230911_70_reg_tc_learn003_pre_powercycle_recheck`
+`result/csk5062_xiaodu_fan/0429230940_71_reg_tc_learn003_powercycle_boot`
+`result/csk5062_xiaodu_fan/0429230959_72_reg_tc_learn003_post_powercycle_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3383,9 +3358,9 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/88_powerloss_during_case_enter_learning`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/89_powerloss_during_case_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/90_powerloss_during_case_recover_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/89_powerloss_during_case_enter_learning`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/90_powerloss_during_case_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/91_powerloss_during_case_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3445,8 +3420,8 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120149_19_reg_voice003_cmd_retry_recover_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120225_20_reg_voice003_cmd_retry_recover_alias_recheck`
+          <t>`result/csk5062_xiaodu_fan/0429225525_19_reg_voice003_cmd_retry_recover_sequence`
+`result/csk5062_xiaodu_fan/0429225601_20_reg_voice003_cmd_retry_recover_alias_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3505,9 +3480,9 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121024_51_reg_voice004_wakeup_retry_recover_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121056_52_reg_voice004_wakeup_retry_recover_recheck_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121107_53_reg_voice004_wakeup_retry_recover_default_wake_ok`
+          <t>`result/csk5062_xiaodu_fan/0429230349_51_reg_voice004_wakeup_retry_recover_sequence`
+`result/csk5062_xiaodu_fan/0429230421_52_reg_voice004_wakeup_retry_recover_recheck_open`
+`result/csk5062_xiaodu_fan/0429230432_53_reg_voice004_wakeup_retry_recover_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3566,8 +3541,8 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120258_23_reg_voice005_cmd_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120343_24_reg_voice005_cmd_retry_exhaust_failed_alias_probe`
+          <t>`result/csk5062_xiaodu_fan/0429225635_23_reg_voice005_cmd_retry_exhaust_sequence`
+`result/csk5062_xiaodu_fan/0429225719_24_reg_voice005_cmd_retry_exhaust_failed_alias_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3626,9 +3601,9 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/97_reg_cfg_wake_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/98_reg_cfg_wake_retry_exhaust_failed_wake_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/99_reg_cfg_wake_retry_exhaust_default_wake_ok`
+          <t>`result/csk5062_xiaodu_fan/0429230505_56_reg_voice006_wakeup_retry_exhaust_sequence`
+`result/csk5062_xiaodu_fan/0429230557_58_reg_voice006_wakeup_retry_exhaust_failed_wake_probe`
+`result/csk5062_xiaodu_fan/0429230612_59_reg_voice006_wakeup_retry_exhaust_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3687,9 +3662,9 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/102_reg_conflict_cmd_volume_word_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/103_reg_conflict_reboot_after_attempt`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/104_reg_conflict_cmd_volume_word_recheck`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/104_reg_conflict_cmd_volume_word_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/105_reg_conflict_reboot_after_attempt`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/106_reg_conflict_cmd_volume_word_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3747,9 +3722,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/25_closure_conflict_default_wake_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/26_closure_conflict_default_wake_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/27_closure_conflict_default_wake_sequence`
+          <t>`result/csk5062_xiaodu_fan/0429230645_62_reg_voice008_wakeup_conflict_default_xiaodu`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3807,7 +3780,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120514_31_reg_voice009_cmd_reserved_learn_wakeup_word`
+          <t>`result/csk5062_xiaodu_fan/0429225850_31_reg_voice009_cmd_reserved_learn_wakeup_word`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3865,7 +3838,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426121349_64_reg_voice010_wakeup_reserved_learn_cmd_word`
+          <t>`result/csk5062_xiaodu_fan/0429230731_65_reg_voice010_wakeup_reserved_learn_cmd_word`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3925,9 +3898,9 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426115953_10_reg_delete_cmd_confirm_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120008_11_reg_delete_cmd_confirm_alias_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120019_12_reg_delete_cmd_confirm_default_close_ok`
+          <t>`result/csk5062_xiaodu_fan/0429225329_10_reg_delete_cmd_confirm_sequence`
+`result/csk5062_xiaodu_fan/0429225344_11_reg_delete_cmd_confirm_alias_blocked`
+`result/csk5062_xiaodu_fan/0429225355_12_reg_delete_cmd_confirm_default_close_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3987,17 +3960,8 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/08_closure_regcmd_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/09_closure_regcmd_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/11_closure_regcmd_retry_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/12_closure_regcmd_retry_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/13_closure_regcmd_learn_close_alias_retry`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/14_closure_regcmd_force_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/15_closure_regcmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/16_closure_regcmd_alias_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/17_closure_regcmd_default_after_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/18_closure_regcmd_delete_exit_keep`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_122152_two_req_xiaodu_closure_r1/03_execution/steps/19_closure_regcmd_alias_after_delete_exit`
+          <t>`result/csk5062_xiaodu_fan/0429225303_08_reg_delete_cmd_exit_keep`
+`result/csk5062_xiaodu_fan/0429225318_09_reg_delete_cmd_exit_keep_alias_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4057,10 +4021,10 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120859_45_reg_voice013_delete_wakeup_confirm_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120918_46_reg_voice013_delete_wakeup_confirm_reboot_after_delete`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120936_47_reg_voice013_delete_wakeup_confirm_learned_wake_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120951_48_reg_voice013_delete_wakeup_confirm_default_wake_ok`
+          <t>`result/csk5062_xiaodu_fan/0429230224_45_reg_voice013_delete_wakeup_confirm_sequence`
+`result/csk5062_xiaodu_fan/0429230243_46_reg_voice013_delete_wakeup_confirm_reboot_after_delete`
+`result/csk5062_xiaodu_fan/0429230301_47_reg_voice013_delete_wakeup_confirm_learned_wake_blocked`
+`result/csk5062_xiaodu_fan/0429230316_48_reg_voice013_delete_wakeup_confirm_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4120,8 +4084,8 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120831_43_reg_voice014_delete_wakeup_exit_keep`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_115731_two_req_xiaodu_voice_reg_r1/steps/0426120848_44_reg_voice014_delete_wakeup_exit_keep_recheck`
+          <t>`result/csk5062_xiaodu_fan/0429230158_43_reg_voice014_delete_wakeup_exit_keep`
+`result/csk5062_xiaodu_fan/0429230212_44_reg_voice014_delete_wakeup_exit_keep_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4173,14 +4137,14 @@
           <t>辅助看 `AGAIN=36dB`、`DGAIN=6dB`</t>
         </is>
       </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>TODO</t>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4240,8 +4204,9 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_121800_two_req_xiaodu_timeout_volume_r1/03_execution/steps/04_probe_wake_only_timeout`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_121800_two_req_xiaodu_timeout_volume_r1/03_execution/steps/06_probe_wake_cmd_timeout`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/23_cfg_wake_timeout_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/24_cfg_wake_timeout_probe_settle`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/25_cfg_wake_timeout_post_command_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4302,21 +4267,21 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/04_cfg_default_volume_position_probe_default_to_max_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/05_cfg_default_volume_position_probe_default_to_max_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/06_cfg_default_volume_position_probe_default_to_max_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/07_cfg_default_volume_position_probe_default_to_max_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/08_cfg_default_volume_position_probe_max_to_min_down_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/09_cfg_default_volume_position_probe_max_to_min_down_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/10_cfg_default_volume_position_probe_max_to_min_down_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/11_cfg_default_volume_position_probe_max_to_min_down_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/12_cfg_default_volume_position_probe_max_to_min_down_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/13_cfg_default_volume_position_probe_min_to_max_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/14_cfg_default_volume_position_probe_min_to_max_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/15_cfg_default_volume_position_probe_min_to_max_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/16_cfg_default_volume_position_probe_min_to_max_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/17_cfg_default_volume_position_probe_min_to_max_up_5`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/04_cfg_default_volume_position_probe_default_to_max_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/05_cfg_default_volume_position_probe_default_to_max_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/06_cfg_default_volume_position_probe_default_to_max_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/07_cfg_default_volume_position_probe_default_to_max_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/08_cfg_default_volume_position_probe_max_to_min_down_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/09_cfg_default_volume_position_probe_max_to_min_down_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/10_cfg_default_volume_position_probe_max_to_min_down_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/11_cfg_default_volume_position_probe_max_to_min_down_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/12_cfg_default_volume_position_probe_max_to_min_down_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/13_cfg_default_volume_position_probe_min_to_max_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/14_cfg_default_volume_position_probe_min_to_max_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/15_cfg_default_volume_position_probe_min_to_max_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/16_cfg_default_volume_position_probe_min_to_max_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/17_cfg_default_volume_position_probe_min_to_max_up_5`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4375,21 +4340,21 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/27_cfg_volume_level_probe_min_anchor`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/28_cfg_volume_level_probe_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/29_cfg_volume_level_probe_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/30_cfg_volume_level_probe_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/31_cfg_volume_level_probe_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/32_cfg_volume_level_probe_up_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/33_cfg_volume_level_probe_max_anchor`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/34_cfg_volume_level_probe_down_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/35_cfg_volume_level_probe_down_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/36_cfg_volume_level_probe_down_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/37_cfg_volume_level_probe_down_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/38_cfg_volume_level_probe_down_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/39_cfg_volume_persist_probe_min`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/40_cfg_volume_persist_wait_refresh`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/41_cfg_volume_powercycle_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/27_cfg_volume_level_probe_min_anchor`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/28_cfg_volume_level_probe_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/29_cfg_volume_level_probe_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/30_cfg_volume_level_probe_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/31_cfg_volume_level_probe_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/32_cfg_volume_level_probe_up_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/33_cfg_volume_level_probe_max_anchor`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/34_cfg_volume_level_probe_down_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/35_cfg_volume_level_probe_down_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/36_cfg_volume_level_probe_down_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/37_cfg_volume_level_probe_down_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/38_cfg_volume_level_probe_down_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/39_cfg_volume_persist_probe_min`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/40_cfg_volume_persist_wait_refresh`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/41_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4448,7 +4413,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/03_assist_gate_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/03_assist_gate_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4508,8 +4473,8 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/48_assist_voice_off_setup`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/51_voice_valid_proto_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/48_assist_voice_off_setup`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/51_voice_valid_proto_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4568,7 +4533,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/26_cfg_passive_report_proto`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/26_cfg_passive_report_proto`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4627,7 +4592,7 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/73_reg_cmd_learn_close_sequence`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/74_reg_cmd_learn_close_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4686,7 +4651,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4745,8 +4710,8 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/93_reg_cfg_cmd_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/94_reg_cfg_cmd_retry_exhaust_failed_alias_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/94_reg_cfg_cmd_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/95_reg_cfg_cmd_retry_exhaust_failed_alias_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4805,9 +4770,10 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/97_reg_cfg_wake_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/98_reg_cfg_wake_retry_exhaust_failed_wake_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/99_reg_cfg_wake_retry_exhaust_default_wake_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/98_reg_cfg_wake_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/99_reg_cfg_wake_retry_after_exhaust_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/100_reg_cfg_wake_retry_exhaust_failed_wake_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/101_reg_cfg_wake_retry_exhaust_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4860,15 +4826,28 @@
           <t>不能用启动 `regCmdCount` 单点推断模板已满；必须有主动填满、保存、重入三段证据</t>
         </is>
       </c>
-      <c r="J72" s="6" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
+      <c r="J72" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/01_assist_startup_powercycle_capture`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/20_assist_reg_cmd_template_full_entry`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/01_regcfg005_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/02_regcfg005_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/03_regcfg005_learn_close_first_01`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/04_regcfg005_learn_close_first_02`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/05_regcfg005_learn_close_first_03`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/06_regcfg005_learn_close_first_04`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/07_regcfg005_learn_close_first_05`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/08_regcfg005_reenter_after_close_01`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/09_regcfg005_reenter_after_close_02`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/10_regcfg005_learn_open_second_01`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/11_regcfg005_learn_open_second_02`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/12_regcfg005_learn_open_second_03`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/13_regcfg005_learn_open_second_04`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/14_regcfg005_reboot_after_fill`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/15_regcfg005_reenter_after_active_fill`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4927,9 +4906,9 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/80_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/81_reg_wake_template_full_reenter`
-`deliverables/csk5062_xiaodu_fan/reports/20260426_111933_two_req_xiaodu_main_r1/03_execution/steps/82_reg_wake_newword_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/82_reg_wake_template_full_reenter`
+`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/83_reg_wake_newword_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4953,12 +4932,12 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>统计项</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>值</t>
         </is>
@@ -4981,7 +4960,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4">
@@ -5001,7 +4980,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -5011,7 +4990,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Add platform profile and Cucumber execution assets
</commit_message>
<xml_diff>
--- a/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
+++ b/deliverables/csk5062_xiaodu_fan/cases/测试用例-正式版.xlsx
@@ -577,7 +577,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -636,8 +636,8 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/02_burn/burn.log`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/02_burn/burn.log`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -696,7 +696,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -755,7 +755,7 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/03_sess_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/03_sess_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -814,7 +814,7 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/04_sess_timeout_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/04_sess_timeout_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -873,8 +873,8 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/04_sess_timeout_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/05_sess_timeout_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/04_sess_timeout_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/05_sess_timeout_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -933,7 +933,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/06_sess_exit_then_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/06_sess_exit_then_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -992,8 +992,8 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/45_sess_exit_sequence_only`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/46_sess_exit_rewake_open_recovery`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/45_sess_exit_sequence_only`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/46_sess_exit_rewake_open_recovery`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/44_sess_idle_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/44_sess_idle_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/03_sess_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/03_sess_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1168,7 +1168,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/07_ctrl_close`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/07_ctrl_close`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/08_ctrl_power_on`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/08_ctrl_power_on`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/09_ctrl_power_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/09_ctrl_power_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1343,7 +1343,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/10_vol_up_down`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/10_vol_up_down`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1402,8 +1402,8 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/11_vol_max`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/12_vol_min`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/11_vol_max`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/12_vol_min`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1463,9 +1463,9 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/39_cfg_volume_persist_probe_min`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/40_cfg_volume_persist_wait_refresh`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/41_cfg_volume_powercycle_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/39_cfg_volume_persist_probe_min`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/40_cfg_volume_persist_wait_refresh`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/41_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1524,7 +1524,7 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/47_volume_rapid_stability`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/47_volume_rapid_stability`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1583,8 +1583,8 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/16_report_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/17_report_off_then_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/16_report_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/17_report_off_then_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1643,9 +1643,9 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/15_report_passive_baseline`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/16_report_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/18_report_passive_after_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/15_report_passive_baseline`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/16_report_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/18_report_passive_after_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1705,9 +1705,9 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/19_report_on_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/20_report_on_then_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/21_report_passive_after_on`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/19_report_on_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/20_report_on_then_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/21_report_passive_after_on`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1766,9 +1766,9 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/22_report_off_before_powercycle`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/23_report_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/24_report_after_powercycle_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/22_report_off_before_powercycle`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/23_report_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/24_report_after_powercycle_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1827,8 +1827,8 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/27_voice_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/28_voice_blocked_after_off`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/27_voice_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/28_voice_blocked_after_off`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1887,8 +1887,8 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/31_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/32_voice_open_after_proto`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/31_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/32_voice_open_after_proto`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -1947,8 +1947,8 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/51_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/52_voice_on_then_volume_up`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/51_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/52_voice_on_then_volume_up`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2007,12 +2007,12 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/27_voice_off_set`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/29_voice_off_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/30_voice_blocked_after_powercycle`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/31_voice_valid_proto_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/33_voice_on_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/34_voice_open_after_powercycle`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/27_voice_off_set`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/29_voice_off_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/30_voice_blocked_after_powercycle`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/31_voice_valid_proto_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/33_voice_on_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/34_voice_open_after_powercycle`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2071,9 +2071,9 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/48_assist_voice_off_setup`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/49_voice_invalid_proto`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/50_voice_invalid_proto_then_wake_open_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/48_assist_voice_off_setup`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/49_voice_invalid_proto`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/50_voice_invalid_proto_then_wake_open_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2132,9 +2132,9 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/38_switch_idle_before_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/39_switch_xiaoai_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/38_switch_idle_before_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/39_switch_xiaoai_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2192,9 +2192,9 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/40_switch_idle_before_default`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/41_switch_default_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/40_switch_idle_before_default`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/41_switch_default_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2252,9 +2252,9 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/62_switch_idle_before_other_wake_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/63_switch_other_wake_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/62_switch_idle_before_other_wake_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/63_switch_other_wake_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2314,11 +2314,11 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/54_switch_idle_before_current_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/55_switch_current_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/56_switch_idle_before_current_wake_volume`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/57_switch_current_wake_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/54_switch_idle_before_current_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/55_switch_current_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/56_switch_idle_before_current_wake_volume`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/57_switch_current_wake_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2378,11 +2378,11 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/58_switch_idle_before_default_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/59_switch_default_wake_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/60_switch_idle_before_default_wake_volume`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/61_switch_default_wake_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/58_switch_idle_before_default_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/59_switch_default_wake_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/60_switch_idle_before_default_wake_volume`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/61_switch_default_wake_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2441,12 +2441,12 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/42_switch_powercycle_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/43_switch_idle_before_xiaoai_after_power`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/44_switch_xiaoai_after_power_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/45_switch_idle_before_default_after_power`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/46_switch_default_after_power_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/37_switch_wake_to_xiaoai`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/42_switch_powercycle_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/43_switch_idle_before_xiaoai_after_power`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/44_switch_xiaoai_after_power_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/45_switch_idle_before_default_after_power`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/46_switch_default_after_power_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2505,11 +2505,11 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/53_switch_wake_to_next`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/64_switch_cycle_to_tmall`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/65_switch_idle_before_tmall_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/66_switch_cycle_tmall_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/67_switch_cycle_back_default`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/53_switch_wake_to_next`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/64_switch_cycle_to_tmall`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/65_switch_idle_before_tmall_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/66_switch_cycle_tmall_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/67_switch_cycle_back_default`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2567,7 +2567,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/49_reg_entry_cmd_only`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/49_reg_entry_cmd_only`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/56_reg_entry_wake_only`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/56_reg_entry_wake_only`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2684,9 +2684,9 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/71_reg_entry_timeout_wait30s`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/72_reg_entry_timeout_idle_30s`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/73_reg_entry_timeout_recover_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/71_reg_entry_timeout_wait30s`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/72_reg_entry_timeout_idle_30s`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/73_reg_entry_timeout_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2745,8 +2745,8 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/52_reg_exit_learning_then_recover`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_224030_xiaodu5062_unified_full_suite_r1_missing_nonreg/03_execution/steps/53_reg_exit_default_open_recover`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/52_reg_exit_learning_then_recover`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_171731_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_missing_nonreg/03_execution/steps/53_reg_exit_default_open_recover`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2805,10 +2805,10 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225133_03_reg_tc_learn_cmd_close_sequence`
-`result/csk5062_xiaodu_fan/0429225206_04_reg_tc_learn_cmd_close_save_closure`
-`result/csk5062_xiaodu_fan/0429225223_05_reg_tc_learn_cmd_close_persist_reboot`
-`result/csk5062_xiaodu_fan/0429225241_06_reg_tc_learn_cmd_close_alias_recheck`
+          <t>`result/csk5062_xiaodu_fan/0514172831_03_reg_tc_learn_cmd_close_sequence`
+`result/csk5062_xiaodu_fan/0514172905_04_reg_tc_learn_cmd_close_save_closure`
+`result/csk5062_xiaodu_fan/0514172922_05_reg_tc_learn_cmd_close_persist_reboot`
+`result/csk5062_xiaodu_fan/0514172940_06_reg_tc_learn_cmd_close_alias_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2867,10 +2867,10 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225133_03_reg_tc_learn_cmd_close_sequence`
-`result/csk5062_xiaodu_fan/0429225206_04_reg_tc_learn_cmd_close_save_closure`
-`result/csk5062_xiaodu_fan/0429225223_05_reg_tc_learn_cmd_close_persist_reboot`
-`result/csk5062_xiaodu_fan/0429225252_07_reg_tc_learn_cmd_close_after_reboot_alias`
+          <t>`result/csk5062_xiaodu_fan/0514172831_03_reg_tc_learn_cmd_close_sequence`
+`result/csk5062_xiaodu_fan/0514172905_04_reg_tc_learn_cmd_close_save_closure`
+`result/csk5062_xiaodu_fan/0514172922_05_reg_tc_learn_cmd_close_persist_reboot`
+`result/csk5062_xiaodu_fan/0514172951_07_reg_tc_learn_cmd_close_after_reboot_alias`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2929,11 +2929,11 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/74_reg_cmd_learn_close_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/75_reg_cmd_learn_close_save_closure`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/76_reg_cmd_reboot_after_save`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/77_reg_cmd_alias_close_recheck`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/78_reg_cmd_default_close_recheck`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/74_reg_cmd_learn_close_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/75_reg_cmd_learn_close_save_closure`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/76_reg_cmd_reboot_after_save`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/77_reg_cmd_alias_close_recheck`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/78_reg_cmd_default_close_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -2992,8 +2992,8 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230044_38_reg_voice002_learn_wakeup_sequence`
-`result/csk5062_xiaodu_fan/0429230106_39_reg_voice002_learned_wake_recheck_open`
+          <t>`result/csk5062_xiaodu_fan/0514173750_38_reg_voice002_learn_wakeup_sequence`
+`result/csk5062_xiaodu_fan/0514173809_39_reg_voice002_learned_wake_recheck_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3051,8 +3051,8 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230044_38_reg_voice002_learn_wakeup_sequence`
-`result/csk5062_xiaodu_fan/0429230117_40_reg_voice002_default_wake_still_open_ok`
+          <t>`result/csk5062_xiaodu_fan/0514173750_38_reg_voice002_learn_wakeup_sequence`
+`result/csk5062_xiaodu_fan/0514173820_40_reg_voice002_default_wake_still_open_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3112,9 +3112,9 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/83_reg_wake_newword_open`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/84_reg_wake_newword_volume`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/83_reg_wake_newword_open`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/84_reg_wake_newword_volume`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3172,9 +3172,9 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/85_reg_wake_idle_before_other_ordinary_blocked`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/86_reg_wake_other_ordinary_blocked`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/85_reg_wake_idle_before_other_ordinary_blocked`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/86_reg_wake_other_ordinary_blocked`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3234,8 +3234,8 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225935_34_reg_tc_learn_prev_boundary`
-`result/csk5062_xiaodu_fan/0429225957_35_reg_tc_learn_next_boundary_full`
+          <t>`result/csk5062_xiaodu_fan/0514173633_34_reg_tc_learn_prev_boundary`
+`result/csk5062_xiaodu_fan/0514173655_35_reg_tc_learn_next_boundary_full`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3295,11 +3295,11 @@
       </c>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230818_68_reg_tc_learn003_learn_wakeup_sequence`
-`result/csk5062_xiaodu_fan/0429230841_69_reg_tc_learn003_learn_cmd_full_sequence`
-`result/csk5062_xiaodu_fan/0429230911_70_reg_tc_learn003_pre_powercycle_recheck`
-`result/csk5062_xiaodu_fan/0429230940_71_reg_tc_learn003_powercycle_boot`
-`result/csk5062_xiaodu_fan/0429230959_72_reg_tc_learn003_post_powercycle_recheck`
+          <t>`result/csk5062_xiaodu_fan/0514174521_68_reg_tc_learn003_learn_wakeup_sequence`
+`result/csk5062_xiaodu_fan/0514174544_69_reg_tc_learn003_learn_cmd_full_sequence`
+`result/csk5062_xiaodu_fan/0514174613_70_reg_tc_learn003_pre_powercycle_recheck`
+`result/csk5062_xiaodu_fan/0514174642_71_reg_tc_learn003_powercycle_boot`
+`result/csk5062_xiaodu_fan/0514174701_72_reg_tc_learn003_post_powercycle_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3358,9 +3358,9 @@
       </c>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/89_powerloss_during_case_enter_learning`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/90_powerloss_during_case_boot`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/91_powerloss_during_case_recover_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/89_powerloss_during_case_enter_learning`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/90_powerloss_during_case_boot`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/91_powerloss_during_case_recover_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3420,8 +3420,8 @@
       </c>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225525_19_reg_voice003_cmd_retry_recover_sequence`
-`result/csk5062_xiaodu_fan/0429225601_20_reg_voice003_cmd_retry_recover_alias_recheck`
+          <t>`result/csk5062_xiaodu_fan/0514173224_19_reg_voice003_cmd_retry_recover_sequence`
+`result/csk5062_xiaodu_fan/0514173300_20_reg_voice003_cmd_retry_recover_alias_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3480,9 +3480,9 @@
       </c>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230349_51_reg_voice004_wakeup_retry_recover_sequence`
-`result/csk5062_xiaodu_fan/0429230421_52_reg_voice004_wakeup_retry_recover_recheck_open`
-`result/csk5062_xiaodu_fan/0429230432_53_reg_voice004_wakeup_retry_recover_default_wake_ok`
+          <t>`result/csk5062_xiaodu_fan/0514174051_51_reg_voice004_wakeup_retry_recover_sequence`
+`result/csk5062_xiaodu_fan/0514174123_52_reg_voice004_wakeup_retry_recover_recheck_open`
+`result/csk5062_xiaodu_fan/0514174134_53_reg_voice004_wakeup_retry_recover_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3541,8 +3541,8 @@
       </c>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225635_23_reg_voice005_cmd_retry_exhaust_sequence`
-`result/csk5062_xiaodu_fan/0429225719_24_reg_voice005_cmd_retry_exhaust_failed_alias_probe`
+          <t>`result/csk5062_xiaodu_fan/0514173333_23_reg_voice005_cmd_retry_exhaust_sequence`
+`result/csk5062_xiaodu_fan/0514173417_24_reg_voice005_cmd_retry_exhaust_failed_alias_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3601,9 +3601,9 @@
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230505_56_reg_voice006_wakeup_retry_exhaust_sequence`
-`result/csk5062_xiaodu_fan/0429230557_58_reg_voice006_wakeup_retry_exhaust_failed_wake_probe`
-`result/csk5062_xiaodu_fan/0429230612_59_reg_voice006_wakeup_retry_exhaust_default_wake_ok`
+          <t>`result/csk5062_xiaodu_fan/0514174208_56_reg_voice006_wakeup_retry_exhaust_sequence`
+`result/csk5062_xiaodu_fan/0514174300_58_reg_voice006_wakeup_retry_exhaust_failed_wake_probe`
+`result/csk5062_xiaodu_fan/0514174315_59_reg_voice006_wakeup_retry_exhaust_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3662,9 +3662,9 @@
       </c>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/104_reg_conflict_cmd_volume_word_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/105_reg_conflict_reboot_after_attempt`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/106_reg_conflict_cmd_volume_word_recheck`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/104_reg_conflict_cmd_volume_word_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/105_reg_conflict_reboot_after_attempt`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/106_reg_conflict_cmd_volume_word_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3722,7 +3722,7 @@
       </c>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230645_62_reg_voice008_wakeup_conflict_default_xiaodu`
+          <t>`result/csk5062_xiaodu_fan/0514174348_62_reg_voice008_wakeup_conflict_default_xiaodu`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3780,7 +3780,7 @@
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225850_31_reg_voice009_cmd_reserved_learn_wakeup_word`
+          <t>`result/csk5062_xiaodu_fan/0514173549_31_reg_voice009_cmd_reserved_learn_wakeup_word`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230731_65_reg_voice010_wakeup_reserved_learn_cmd_word`
+          <t>`result/csk5062_xiaodu_fan/0514174434_65_reg_voice010_wakeup_reserved_learn_cmd_word`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3898,9 +3898,9 @@
       </c>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225329_10_reg_delete_cmd_confirm_sequence`
-`result/csk5062_xiaodu_fan/0429225344_11_reg_delete_cmd_confirm_alias_blocked`
-`result/csk5062_xiaodu_fan/0429225355_12_reg_delete_cmd_confirm_default_close_ok`
+          <t>`result/csk5062_xiaodu_fan/0514173027_10_reg_delete_cmd_confirm_sequence`
+`result/csk5062_xiaodu_fan/0514173042_11_reg_delete_cmd_confirm_alias_blocked`
+`result/csk5062_xiaodu_fan/0514173053_12_reg_delete_cmd_confirm_default_close_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -3960,8 +3960,8 @@
       </c>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429225303_08_reg_delete_cmd_exit_keep`
-`result/csk5062_xiaodu_fan/0429225318_09_reg_delete_cmd_exit_keep_alias_recheck`
+          <t>`result/csk5062_xiaodu_fan/0514173002_08_reg_delete_cmd_exit_keep`
+`result/csk5062_xiaodu_fan/0514173016_09_reg_delete_cmd_exit_keep_alias_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4021,10 +4021,10 @@
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230224_45_reg_voice013_delete_wakeup_confirm_sequence`
-`result/csk5062_xiaodu_fan/0429230243_46_reg_voice013_delete_wakeup_confirm_reboot_after_delete`
-`result/csk5062_xiaodu_fan/0429230301_47_reg_voice013_delete_wakeup_confirm_learned_wake_blocked`
-`result/csk5062_xiaodu_fan/0429230316_48_reg_voice013_delete_wakeup_confirm_default_wake_ok`
+          <t>`result/csk5062_xiaodu_fan/0514173926_45_reg_voice013_delete_wakeup_confirm_sequence`
+`result/csk5062_xiaodu_fan/0514173945_46_reg_voice013_delete_wakeup_confirm_reboot_after_delete`
+`result/csk5062_xiaodu_fan/0514174003_47_reg_voice013_delete_wakeup_confirm_learned_wake_blocked`
+`result/csk5062_xiaodu_fan/0514174018_48_reg_voice013_delete_wakeup_confirm_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4084,8 +4084,8 @@
       </c>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>`result/csk5062_xiaodu_fan/0429230158_43_reg_voice014_delete_wakeup_exit_keep`
-`result/csk5062_xiaodu_fan/0429230212_44_reg_voice014_delete_wakeup_exit_keep_recheck`
+          <t>`result/csk5062_xiaodu_fan/0514173900_43_reg_voice014_delete_wakeup_exit_keep`
+`result/csk5062_xiaodu_fan/0514173915_44_reg_voice014_delete_wakeup_exit_keep_recheck`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4144,7 +4144,7 @@
       </c>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4204,9 +4204,9 @@
       </c>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/23_cfg_wake_timeout_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/24_cfg_wake_timeout_probe_settle`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/25_cfg_wake_timeout_post_command_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/23_cfg_wake_timeout_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/24_cfg_wake_timeout_probe_settle`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/25_cfg_wake_timeout_post_command_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4267,21 +4267,21 @@
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/04_cfg_default_volume_position_probe_default_to_max_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/05_cfg_default_volume_position_probe_default_to_max_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/06_cfg_default_volume_position_probe_default_to_max_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/07_cfg_default_volume_position_probe_default_to_max_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/08_cfg_default_volume_position_probe_max_to_min_down_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/09_cfg_default_volume_position_probe_max_to_min_down_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/10_cfg_default_volume_position_probe_max_to_min_down_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/11_cfg_default_volume_position_probe_max_to_min_down_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/12_cfg_default_volume_position_probe_max_to_min_down_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/13_cfg_default_volume_position_probe_min_to_max_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/14_cfg_default_volume_position_probe_min_to_max_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/15_cfg_default_volume_position_probe_min_to_max_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/16_cfg_default_volume_position_probe_min_to_max_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/17_cfg_default_volume_position_probe_min_to_max_up_5`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/01_assist_startup_powercycle_capture`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/04_cfg_default_volume_position_probe_default_to_max_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/05_cfg_default_volume_position_probe_default_to_max_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/06_cfg_default_volume_position_probe_default_to_max_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/07_cfg_default_volume_position_probe_default_to_max_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/08_cfg_default_volume_position_probe_max_to_min_down_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/09_cfg_default_volume_position_probe_max_to_min_down_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/10_cfg_default_volume_position_probe_max_to_min_down_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/11_cfg_default_volume_position_probe_max_to_min_down_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/12_cfg_default_volume_position_probe_max_to_min_down_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/13_cfg_default_volume_position_probe_min_to_max_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/14_cfg_default_volume_position_probe_min_to_max_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/15_cfg_default_volume_position_probe_min_to_max_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/16_cfg_default_volume_position_probe_min_to_max_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/17_cfg_default_volume_position_probe_min_to_max_up_5`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4340,21 +4340,21 @@
       </c>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/27_cfg_volume_level_probe_min_anchor`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/28_cfg_volume_level_probe_up_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/29_cfg_volume_level_probe_up_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/30_cfg_volume_level_probe_up_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/31_cfg_volume_level_probe_up_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/32_cfg_volume_level_probe_up_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/33_cfg_volume_level_probe_max_anchor`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/34_cfg_volume_level_probe_down_1`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/35_cfg_volume_level_probe_down_2`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/36_cfg_volume_level_probe_down_3`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/37_cfg_volume_level_probe_down_4`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/38_cfg_volume_level_probe_down_5`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/39_cfg_volume_persist_probe_min`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/40_cfg_volume_persist_wait_refresh`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/41_cfg_volume_powercycle_reboot`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/27_cfg_volume_level_probe_min_anchor`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/28_cfg_volume_level_probe_up_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/29_cfg_volume_level_probe_up_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/30_cfg_volume_level_probe_up_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/31_cfg_volume_level_probe_up_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/32_cfg_volume_level_probe_up_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/33_cfg_volume_level_probe_max_anchor`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/34_cfg_volume_level_probe_down_1`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/35_cfg_volume_level_probe_down_2`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/36_cfg_volume_level_probe_down_3`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/37_cfg_volume_level_probe_down_4`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/38_cfg_volume_level_probe_down_5`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/39_cfg_volume_persist_probe_min`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/40_cfg_volume_persist_wait_refresh`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/41_cfg_volume_powercycle_reboot`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4413,7 +4413,7 @@
       </c>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/03_assist_gate_default_wake_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/03_assist_gate_default_wake_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4473,8 +4473,8 @@
       </c>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/48_assist_voice_off_setup`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/51_voice_valid_proto_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/48_assist_voice_off_setup`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/51_voice_valid_proto_open`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4533,7 +4533,7 @@
       </c>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/26_cfg_passive_report_proto`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/26_cfg_passive_report_proto`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/74_reg_cmd_learn_close_sequence`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/74_reg_cmd_learn_close_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4710,8 +4710,8 @@
       </c>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/94_reg_cfg_cmd_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/95_reg_cfg_cmd_retry_exhaust_failed_alias_probe`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/94_reg_cfg_cmd_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/95_reg_cfg_cmd_retry_exhaust_failed_alias_probe`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4770,10 +4770,10 @@
       </c>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/98_reg_cfg_wake_retry_exhaust_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/99_reg_cfg_wake_retry_after_exhaust_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/100_reg_cfg_wake_retry_exhaust_failed_wake_probe`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/101_reg_cfg_wake_retry_exhaust_default_wake_ok`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/98_reg_cfg_wake_retry_exhaust_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/99_reg_cfg_wake_retry_after_exhaust_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/100_reg_cfg_wake_retry_exhaust_failed_wake_probe`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/101_reg_cfg_wake_retry_exhaust_default_wake_ok`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4833,21 +4833,21 @@
       </c>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/01_regcfg005_config_clear`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/02_regcfg005_reboot`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/03_regcfg005_learn_close_first_01`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/04_regcfg005_learn_close_first_02`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/05_regcfg005_learn_close_first_03`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/06_regcfg005_learn_close_first_04`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/07_regcfg005_learn_close_first_05`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/08_regcfg005_reenter_after_close_01`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/09_regcfg005_reenter_after_close_02`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/10_regcfg005_learn_open_second_01`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/11_regcfg005_learn_open_second_02`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/12_regcfg005_learn_open_second_03`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/13_regcfg005_learn_open_second_04`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/14_regcfg005_reboot_after_fill`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_231733_xiaodu5062_unified_full_suite_r1_regcfg005_closure_r3/03_execution/steps/15_regcfg005_reenter_after_active_fill`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/01_regcfg005_config_clear`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/02_regcfg005_reboot`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/03_regcfg005_learn_close_first_01`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/04_regcfg005_learn_close_first_02`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/05_regcfg005_learn_close_first_03`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/06_regcfg005_learn_close_first_04`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/07_regcfg005_learn_close_first_05`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/08_regcfg005_reenter_after_close_01`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/09_regcfg005_reenter_after_close_02`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/10_regcfg005_learn_open_second_01`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/11_regcfg005_learn_open_second_02`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/12_regcfg005_learn_open_second_03`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/13_regcfg005_learn_open_second_04`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/14_regcfg005_reboot_after_fill`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_174730_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_regcfg005_closure/03_execution/steps/15_regcfg005_reenter_after_active_fill`
 目录重构后复跑闭环</t>
         </is>
       </c>
@@ -4906,9 +4906,9 @@
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/82_reg_wake_template_full_reenter`
-`deliverables/csk5062_xiaodu_fan/reports/20260429_221705_xiaodu5062_unified_full_suite_r1_main_fullflow/03_execution/steps/83_reg_wake_newword_open`
+          <t>`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/81_reg_wake_learn_sequence`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/82_reg_wake_template_full_reenter`
+`deliverables/csk5062_xiaodu_fan/reports/20260514_165414_xiaodu5062_cucumber_all_native_cfgvol_r3_formal_72_inner_formal_main_fullflow/03_execution/steps/83_reg_wake_newword_open`
 目录重构后复跑闭环</t>
         </is>
       </c>

</xml_diff>